<commit_message>
add 2 second to time error, add 1 sec to timeout
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -19,57 +19,25 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Date</t>
   </si>
   <si>
     <t>Question</t>
   </si>
-  <si>
-    <t xml:space="preserve">Вопрос 12: В книге "Час быка" Иван Ефремов упоминает, что на столе у правителя-тирана Чойо Чагаса находилась символическая скульптура, изображающая ИХ. Мы не спрашиваем у вас, что делает или чего не делает каждая из НИХ. Назовите ИХ двумя словами.
-Ответ: Три обезьяны.
-Комментарий: Одна обезьяна заткнула уши, другая закрыла глаза, третья прикрыла рот — одна из обезьян ничего не слышит, вторая ничего не видит, третья ничего не говорит.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вопрос 13: По одной из версий, у вынужденных переселенцев ОН стал аналогом проворной и сообразительной карликовой антилопы. Назовите ЕГО двумя словами.
-Ответ: Братец Кролик.
-Комментарий: Как и другие персонажи "Сказок дядюшки Римуса", хитроумный Братец Кролик является героем фольклора невольников-африканцев. Некоторые исследователи полагали, что в оригинальных африканских сказках роль трИкстера выполняла карликовая антилопа. Поскольку такое животное в Северной Америке не водилось, в фольклоре рабов трИкстером стал кролик.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вопрос 9: Известный русский писатель вспоминал, как одному соседскому старику, "зажившемуся за семьдесят", нетерпеливая невестка влила в ухо кипящий сургуч. Какое произведение возникло под впечатлением от этого случая?
-Ответ: "Леди Макбет Мценского уезда".
-Комментарий: Похожим образом был убит отец Гамлета. Этот случай навел Н.С. Лескова на мысль о том, что и в русских селениях возможны шекспировские страсти.
-</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
   </fonts>
   <fills count="2">
@@ -80,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -88,41 +56,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -133,17 +71,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -430,7 +373,7 @@
     <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -438,48 +381,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="199.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
-      <c r="B2" s="4">
-        <v>45722</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>4</v>
-      </c>
       <c r="E2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="252" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
-        <v>45722</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="1">
+      <c r="E3" s="1" t="str">
         <f ca="1">IF(ISTEXT(INDIRECT(ADDRESS(ROW(),3))),MAX(E2,E1) + 1,"-")</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="212.4" thickBot="1" x14ac:dyDescent="0.35">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
-        <v>45722</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" s="1">
+      <c r="E4" s="1" t="str">
         <f t="shared" ref="E4:E67" ca="1" si="0">IF(ISTEXT(INDIRECT(ADDRESS(ROW(),3))),MAX(E3,E2) + 1,"-")</f>
-        <v>3</v>
+        <v>-</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1491,6 +1416,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="break">
+      <formula>NOT(ISERROR(SEARCH("break",C1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>